<commit_message>
Working code with rate card
All working
</commit_message>
<xml_diff>
--- a/Ref docs/Client Request Details.xlsx
+++ b/Ref docs/Client Request Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{337C324A-460A-4E1A-B2BD-092CDDFF9CA6}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F15341E-AF45-469E-9549-A04DDBEBE847}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="59">
   <si>
     <t>Description</t>
   </si>
@@ -228,6 +228,36 @@
   </si>
   <si>
     <t>Date Raised</t>
+  </si>
+  <si>
+    <t>B-134</t>
+  </si>
+  <si>
+    <t>B-135</t>
+  </si>
+  <si>
+    <t>B-136</t>
+  </si>
+  <si>
+    <t>B-137</t>
+  </si>
+  <si>
+    <t>B-138</t>
+  </si>
+  <si>
+    <t>B-139</t>
+  </si>
+  <si>
+    <t>B-140</t>
+  </si>
+  <si>
+    <t>B-141</t>
+  </si>
+  <si>
+    <t>B-142</t>
+  </si>
+  <si>
+    <t>B-143</t>
   </si>
 </sst>
 </file>
@@ -300,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
@@ -320,10 +350,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -664,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5" style="5" bestFit="1" customWidth="1"/>
@@ -953,8 +979,235 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="8"/>
+    <row r="13" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Working code - Landing and internal pages rewamped
All working
</commit_message>
<xml_diff>
--- a/Ref docs/Client Request Details.xlsx
+++ b/Ref docs/Client Request Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F15341E-AF45-469E-9549-A04DDBEBE847}"/>
+  <xr:revisionPtr revIDLastSave="434" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56AC4CC2-3C55-4C5D-B2BF-058A86024013}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="64">
   <si>
     <t>Description</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t xml:space="preserve">1 resource - FE role </t>
-  </si>
-  <si>
-    <t>Accepted by Staffing Team</t>
   </si>
   <si>
     <t xml:space="preserve">1 resource - FE role - To be offboarded </t>
@@ -259,11 +256,32 @@
   <si>
     <t>B-143</t>
   </si>
+  <si>
+    <t xml:space="preserve">Onboarding </t>
+  </si>
+  <si>
+    <t>Offboarding</t>
+  </si>
+  <si>
+    <t>Resource Demand</t>
+  </si>
+  <si>
+    <t>1 resource - FE role - To be onboarded</t>
+  </si>
+  <si>
+    <t>Request Type</t>
+  </si>
+  <si>
+    <t>Accepted</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-24009]m/d/yyyy;@"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -330,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
@@ -351,6 +369,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,523 +709,590 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="24" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.9140625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="10.9140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.6640625" style="5"/>
+    <col min="2" max="2" width="13.9140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="24" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.9140625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="10.9140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.6640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2" s="8">
+        <v>45306</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H3" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H4" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H5" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H6" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>11</v>
+      <c r="B7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H7" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>11</v>
+      <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H8" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>35</v>
+      <c r="B9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>35</v>
+      <c r="D11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H11" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="H14" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="H15" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="H16" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="H17" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="H18" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="H19" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="H20" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="H21" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F21" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>44</v>
+      <c r="H22" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>